<commit_message>
copy(values): 7つの判断基準の表示順を変更（Self Driven/Challenge/Better Everyday/Legacy/Purpose/Co-Create/Build Systems）＋マスター同期
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YNtH9gBRMgJ8dSqqA3kACx
</commit_message>
<xml_diff>
--- a/docs/web-copy-master.xlsx
+++ b/docs/web-copy-master.xlsx
@@ -6171,7 +6171,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-07</t>
+          <t>ABOUT-VALUES-09</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>Legacy：100年後に、誇れる選択を。</t>
+          <t>Self Driven：自分ごとで動こう。</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
@@ -6213,7 +6213,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-08</t>
+          <t>ABOUT-VALUES-10</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Purpose：目的から、考えよう。</t>
+          <t>Challenge：まず、やってみよう。</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
@@ -6255,7 +6255,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-09</t>
+          <t>ABOUT-VALUES-12</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Self Driven：自分ごとで動こう。</t>
+          <t>Better Everyday：昨日より、少しずつ良くしよう。</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
@@ -6297,7 +6297,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-10</t>
+          <t>ABOUT-VALUES-07</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Challenge：まず、やってみよう。</t>
+          <t>Legacy：100年後に、誇れる選択を。</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
@@ -6339,7 +6339,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-11</t>
+          <t>ABOUT-VALUES-08</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Co-Create：違いを力に、共に創ろう。</t>
+          <t>Purpose：目的から、考えよう。</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
@@ -6381,7 +6381,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-12</t>
+          <t>ABOUT-VALUES-11</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Better Everyday：昨日より、少しずつ良くしよう。</t>
+          <t>Co-Create：違いを力に、共に創ろう。</t>
         </is>
       </c>
       <c r="F101" s="4" t="inlineStr">
@@ -12279,7 +12279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12405,6 +12405,38 @@
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Moments Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>ABOUT-VALUES(判断基準)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Legacy→Purpose→Self Driven→Challenge→Co-Create→Better Everyday→Build Systems</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Self Driven→Challenge→Better Everyday→Legacy→Purpose→Co-Create→Build Systems</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>7つの判断基準の表示順を変更</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Moments Share</t>
         </is>
@@ -15532,7 +15564,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-07</t>
+          <t>ABOUT-VALUES-09</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -15547,7 +15579,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Legacy：100年後に、誇れる選択を。</t>
+          <t>Self Driven：自分ごとで動こう。</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -15569,7 +15601,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-08</t>
+          <t>ABOUT-VALUES-10</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -15584,7 +15616,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Purpose：目的から、考えよう。</t>
+          <t>Challenge：まず、やってみよう。</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -15606,7 +15638,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-09</t>
+          <t>ABOUT-VALUES-12</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -15621,7 +15653,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Self Driven：自分ごとで動こう。</t>
+          <t>Better Everyday：昨日より、少しずつ良くしよう。</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -15643,7 +15675,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-10</t>
+          <t>ABOUT-VALUES-07</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -15658,7 +15690,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Challenge：まず、やってみよう。</t>
+          <t>Legacy：100年後に、誇れる選択を。</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -15680,7 +15712,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-11</t>
+          <t>ABOUT-VALUES-08</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -15695,7 +15727,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Co-Create：違いを力に、共に創ろう。</t>
+          <t>Purpose：目的から、考えよう。</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -15717,7 +15749,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ABOUT-VALUES-12</t>
+          <t>ABOUT-VALUES-11</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -15732,7 +15764,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Better Everyday：昨日より、少しずつ良くしよう。</t>
+          <t>Co-Create：違いを力に、共に創ろう。</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">

</xml_diff>